<commit_message>
Hide Excel data store banner from modal and enhance Firebase export script
</commit_message>
<xml_diff>
--- a/src/data/birthday_wishes.xlsx
+++ b/src/data/birthday_wishes.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:H2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="22.83203125" customWidth="1"/>
@@ -405,7 +405,8 @@
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
     <col min="5" max="5" width="15.83203125" customWidth="1"/>
     <col min="6" max="6" width="60.83203125" customWidth="1"/>
-    <col min="7" max="7" width="12.83203125" customWidth="1"/>
+    <col min="7" max="7" width="10.83203125" customWidth="1"/>
+    <col min="8" max="8" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -428,6 +429,9 @@
         <v>Birthday Message</v>
       </c>
       <c r="G1" t="str">
+        <v>Likes</v>
+      </c>
+      <c r="H1" t="str">
         <v>Status</v>
       </c>
     </row>
@@ -436,7 +440,7 @@
         <v>WISH-001</v>
       </c>
       <c r="B2" t="str">
-        <v>23/9/2026, 12:19:59 am</v>
+        <v>23/9/2026, 12:34:55 am</v>
       </c>
       <c r="C2" t="str">
         <v>Sample Friend</v>
@@ -450,13 +454,16 @@
       <c r="F2" t="str">
         <v>Happy Birthday Klint! Wishing you more success, happiness, and clean code ahead! 🚀</v>
       </c>
-      <c r="G2" t="str">
+      <c r="G2">
+        <v>1</v>
+      </c>
+      <c r="H2" t="str">
         <v>Received</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>